<commit_message>
Tsunami: La Unidad 15-4 Black Bulls ya cuenta en la tabla y en los numeros (jornada 3)
</commit_message>
<xml_diff>
--- a/tsunami-numeros.xlsx
+++ b/tsunami-numeros.xlsx
@@ -469,7 +469,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B25"/>
+  <dimension ref="A1:B24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -483,7 +483,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -532,7 +531,6 @@
         </is>
       </c>
     </row>
-    <row r="7"/>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
@@ -684,7 +682,6 @@
         </is>
       </c>
     </row>
-    <row r="21"/>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
@@ -697,26 +694,13 @@
         </is>
       </c>
     </row>
-    <row r="23"/>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Suspendido</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
-        <is>
-          <t>La Unidad 15-4 Black Bulls (27 sep) terminó, pero en GameChanger quedó abierto del lado de La Unidad. La tabla oficial todavía no lo cuenta y los números de La Unidad siguen como después de la jornada 2; los de Black Bulls ya lo incluyen. Se actualiza cuando el juego se cierre en GameChanger.</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="2" t="inlineStr">
-        <is>
-          <t>Suspendido</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
         <is>
           <t>Piratas vs Elite (27 sep, 1:30 pm) se suspendió por lluvia en la 2.ª entrada. No es válido y se reprograma.</t>
         </is>
@@ -10427,7 +10411,7 @@
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>Black Bulls</t>
+          <t>La Unidad</t>
         </is>
       </c>
       <c r="B12" s="5" t="n">
@@ -10450,13 +10434,13 @@
         </is>
       </c>
       <c r="G12" s="5" t="n">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="H12" s="5" t="n">
-        <v>31</v>
+        <v>19</v>
       </c>
       <c r="I12" s="5" t="n">
-        <v>-14</v>
+        <v>0</v>
       </c>
       <c r="J12" s="5" t="inlineStr">
         <is>
@@ -10527,21 +10511,21 @@
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>La Unidad</t>
+          <t>Black Bulls</t>
         </is>
       </c>
       <c r="B14" s="5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C14" s="5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D14" s="5" t="n">
         <v>0</v>
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t>0.000</t>
+          <t>0.333</t>
         </is>
       </c>
       <c r="F14" s="5" t="inlineStr">
@@ -10550,13 +10534,13 @@
         </is>
       </c>
       <c r="G14" s="5" t="n">
-        <v>4</v>
+        <v>21</v>
       </c>
       <c r="H14" s="5" t="n">
-        <v>15</v>
+        <v>46</v>
       </c>
       <c r="I14" s="5" t="n">
-        <v>-11</v>
+        <v>-25</v>
       </c>
       <c r="J14" s="5" t="inlineStr">
         <is>
@@ -10565,12 +10549,12 @@
       </c>
       <c r="K14" s="5" t="inlineStr">
         <is>
-          <t>0-1</t>
+          <t>0-2</t>
         </is>
       </c>
       <c r="L14" s="5" t="inlineStr">
         <is>
-          <t>0-0</t>
+          <t>1-0</t>
         </is>
       </c>
     </row>
@@ -21376,7 +21360,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N15"/>
+  <dimension ref="A1:N23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -21472,7 +21456,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Selecta Rooki</t>
+          <t>Daryl Him</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -21484,10 +21468,10 @@
         <v>1</v>
       </c>
       <c r="D5" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E5" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F5" t="n">
         <v>0</v>
@@ -21499,11 +21483,11 @@
         <v>0</v>
       </c>
       <c r="I5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>1.000</t>
+          <t>.750</t>
         </is>
       </c>
     </row>
@@ -21548,7 +21532,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Jair Varela</t>
+          <t>Ricardo Martin</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -21566,7 +21550,7 @@
         <v>2</v>
       </c>
       <c r="F7" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G7" t="n">
         <v>0</v>
@@ -21575,7 +21559,7 @@
         <v>0</v>
       </c>
       <c r="I7" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J7" t="inlineStr">
         <is>
@@ -21586,7 +21570,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Euri VALDES</t>
+          <t>Andres Samudio</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -21601,7 +21585,7 @@
         <v>3</v>
       </c>
       <c r="E8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F8" t="n">
         <v>0</v>
@@ -21617,30 +21601,14 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>.333</t>
-        </is>
-      </c>
-      <c r="K8" t="inlineStr">
-        <is>
-          <t>3.2</t>
-        </is>
-      </c>
-      <c r="L8" t="n">
-        <v>0</v>
-      </c>
-      <c r="M8" t="n">
-        <v>0</v>
-      </c>
-      <c r="N8" t="inlineStr">
-        <is>
-          <t>11.45</t>
+          <t>.667</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Sebastiàn Solís</t>
+          <t>Jair Varela</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -21649,29 +21617,29 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D9" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="E9" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G9" t="n">
         <v>0</v>
       </c>
       <c r="H9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I9" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>.333</t>
+          <t>.667</t>
         </is>
       </c>
     </row>
@@ -21687,36 +21655,36 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D10" t="n">
+        <v>6</v>
+      </c>
+      <c r="E10" t="n">
         <v>3</v>
       </c>
-      <c r="E10" t="n">
-        <v>1</v>
-      </c>
       <c r="F10" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G10" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H10" t="n">
         <v>0</v>
       </c>
       <c r="I10" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>.333</t>
+          <t>.600</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Mario Cruz</t>
+          <t>Eduardo Rodriguez</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -21728,13 +21696,13 @@
         <v>1</v>
       </c>
       <c r="D11" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E11" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G11" t="n">
         <v>0</v>
@@ -21743,18 +21711,18 @@
         <v>0</v>
       </c>
       <c r="I11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>.000</t>
+          <t>.500</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>José Acha Castillo</t>
+          <t>Sotolongo</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -21769,10 +21737,10 @@
         <v>2</v>
       </c>
       <c r="E12" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F12" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G12" t="n">
         <v>0</v>
@@ -21781,18 +21749,18 @@
         <v>0</v>
       </c>
       <c r="I12" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>.000</t>
+          <t>.500</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Luis Marin</t>
+          <t>Oscar Ruyery</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -21804,10 +21772,10 @@
         <v>1</v>
       </c>
       <c r="D13" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E13" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F13" t="n">
         <v>0</v>
@@ -21816,118 +21784,428 @@
         <v>0</v>
       </c>
       <c r="H13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>.000</t>
-        </is>
-      </c>
-      <c r="K13" t="inlineStr">
-        <is>
-          <t>2.1</t>
-        </is>
-      </c>
-      <c r="L13" t="n">
-        <v>0</v>
-      </c>
-      <c r="M13" t="n">
-        <v>0</v>
-      </c>
-      <c r="N13" t="inlineStr">
-        <is>
-          <t>24.00</t>
+          <t>.500</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
+          <t>Carlos Hernandez</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>La Unidad</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>1</v>
+      </c>
+      <c r="D14" t="n">
+        <v>2</v>
+      </c>
+      <c r="E14" t="n">
+        <v>1</v>
+      </c>
+      <c r="F14" t="n">
+        <v>0</v>
+      </c>
+      <c r="G14" t="n">
+        <v>0</v>
+      </c>
+      <c r="H14" t="n">
+        <v>0</v>
+      </c>
+      <c r="I14" t="n">
+        <v>1</v>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>.500</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Euri VALDES</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>La Unidad</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>2</v>
+      </c>
+      <c r="D15" t="n">
+        <v>6</v>
+      </c>
+      <c r="E15" t="n">
+        <v>2</v>
+      </c>
+      <c r="F15" t="n">
+        <v>0</v>
+      </c>
+      <c r="G15" t="n">
+        <v>0</v>
+      </c>
+      <c r="H15" t="n">
+        <v>0</v>
+      </c>
+      <c r="I15" t="n">
+        <v>1</v>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>.333</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>3.2</t>
+        </is>
+      </c>
+      <c r="L15" t="n">
+        <v>0</v>
+      </c>
+      <c r="M15" t="n">
+        <v>0</v>
+      </c>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>11.45</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Sebastiàn Solís</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>La Unidad</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>1</v>
+      </c>
+      <c r="D16" t="n">
+        <v>3</v>
+      </c>
+      <c r="E16" t="n">
+        <v>1</v>
+      </c>
+      <c r="F16" t="n">
+        <v>0</v>
+      </c>
+      <c r="G16" t="n">
+        <v>0</v>
+      </c>
+      <c r="H16" t="n">
+        <v>1</v>
+      </c>
+      <c r="I16" t="n">
+        <v>2</v>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>.333</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Selecta Rooki</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>La Unidad</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>2</v>
+      </c>
+      <c r="D17" t="n">
+        <v>4</v>
+      </c>
+      <c r="E17" t="n">
+        <v>1</v>
+      </c>
+      <c r="F17" t="n">
+        <v>0</v>
+      </c>
+      <c r="G17" t="n">
+        <v>0</v>
+      </c>
+      <c r="H17" t="n">
+        <v>0</v>
+      </c>
+      <c r="I17" t="n">
+        <v>0</v>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>.333</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Mario Cruz</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>La Unidad</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>2</v>
+      </c>
+      <c r="D18" t="n">
+        <v>5</v>
+      </c>
+      <c r="E18" t="n">
+        <v>1</v>
+      </c>
+      <c r="F18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G18" t="n">
+        <v>0</v>
+      </c>
+      <c r="H18" t="n">
+        <v>0</v>
+      </c>
+      <c r="I18" t="n">
+        <v>1</v>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>.200</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>José Acha Castillo</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>La Unidad</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>2</v>
+      </c>
+      <c r="D19" t="n">
+        <v>3</v>
+      </c>
+      <c r="E19" t="n">
+        <v>0</v>
+      </c>
+      <c r="F19" t="n">
+        <v>0</v>
+      </c>
+      <c r="G19" t="n">
+        <v>0</v>
+      </c>
+      <c r="H19" t="n">
+        <v>0</v>
+      </c>
+      <c r="I19" t="n">
+        <v>2</v>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>.000</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Luis Marin</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>La Unidad</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>1</v>
+      </c>
+      <c r="D20" t="n">
+        <v>2</v>
+      </c>
+      <c r="E20" t="n">
+        <v>0</v>
+      </c>
+      <c r="F20" t="n">
+        <v>0</v>
+      </c>
+      <c r="G20" t="n">
+        <v>0</v>
+      </c>
+      <c r="H20" t="n">
+        <v>0</v>
+      </c>
+      <c r="I20" t="n">
+        <v>0</v>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>.000</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>2.1</t>
+        </is>
+      </c>
+      <c r="L20" t="n">
+        <v>0</v>
+      </c>
+      <c r="M20" t="n">
+        <v>0</v>
+      </c>
+      <c r="N20" t="inlineStr">
+        <is>
+          <t>24.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
           <t>Leonel González</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
+      <c r="B21" t="inlineStr">
         <is>
           <t>La Unidad</t>
         </is>
       </c>
-      <c r="C14" t="n">
-        <v>1</v>
-      </c>
-      <c r="D14" t="n">
+      <c r="C21" t="n">
+        <v>1</v>
+      </c>
+      <c r="D21" t="n">
         <v>3</v>
       </c>
-      <c r="E14" t="n">
-        <v>0</v>
-      </c>
-      <c r="F14" t="n">
-        <v>0</v>
-      </c>
-      <c r="G14" t="n">
-        <v>0</v>
-      </c>
-      <c r="H14" t="n">
-        <v>0</v>
-      </c>
-      <c r="I14" t="n">
-        <v>0</v>
-      </c>
-      <c r="J14" t="inlineStr">
+      <c r="E21" t="n">
+        <v>0</v>
+      </c>
+      <c r="F21" t="n">
+        <v>0</v>
+      </c>
+      <c r="G21" t="n">
+        <v>0</v>
+      </c>
+      <c r="H21" t="n">
+        <v>0</v>
+      </c>
+      <c r="I21" t="n">
+        <v>0</v>
+      </c>
+      <c r="J21" t="inlineStr">
         <is>
           <t>.000</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="2" t="inlineStr">
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Tomas Scott</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>La Unidad</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>6.0</t>
+        </is>
+      </c>
+      <c r="L22" t="n">
+        <v>1</v>
+      </c>
+      <c r="M22" t="n">
+        <v>1</v>
+      </c>
+      <c r="N22" t="inlineStr">
+        <is>
+          <t>3.500</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
         <is>
           <t>Total del equipo</t>
         </is>
       </c>
-      <c r="B15" s="2" t="n"/>
-      <c r="C15" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="D15" s="2" t="n">
-        <v>26</v>
-      </c>
-      <c r="E15" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="F15" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="G15" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="H15" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="I15" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="J15" s="2" t="inlineStr">
-        <is>
-          <t>.320</t>
-        </is>
-      </c>
-      <c r="K15" s="2" t="inlineStr">
-        <is>
-          <t>6.0</t>
-        </is>
-      </c>
-      <c r="L15" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M15" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="N15" s="2" t="inlineStr">
-        <is>
-          <t>16.33</t>
+      <c r="B23" s="2" t="n"/>
+      <c r="C23" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D23" s="2" t="n">
+        <v>64</v>
+      </c>
+      <c r="E23" s="2" t="n">
+        <v>27</v>
+      </c>
+      <c r="F23" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="G23" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="H23" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="I23" s="2" t="n">
+        <v>18</v>
+      </c>
+      <c r="J23" s="2" t="inlineStr">
+        <is>
+          <t>.443</t>
+        </is>
+      </c>
+      <c r="K23" s="2" t="inlineStr">
+        <is>
+          <t>12.0</t>
+        </is>
+      </c>
+      <c r="L23" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="M23" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="N23" s="2" t="inlineStr">
+        <is>
+          <t>9.917</t>
         </is>
       </c>
     </row>

</xml_diff>